<commit_message>
READY: USD to ARS
</commit_message>
<xml_diff>
--- a/web_parsers/mercado_libre_parser/products.xlsx
+++ b/web_parsers/mercado_libre_parser/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E287"/>
+  <dimension ref="A1:E442"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>13702</v>
+        <v>14936</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>98231</v>
+        <v>93756</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
@@ -5055,7 +5055,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>15078</v>
+        <v>16290</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
@@ -5105,7 +5105,7 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>90326</v>
+        <v>90426</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
@@ -5205,7 +5205,7 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>14095</v>
+        <v>15312</v>
       </c>
       <c r="D192" t="inlineStr">
         <is>
@@ -5280,7 +5280,7 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>90169</v>
+        <v>89680</v>
       </c>
       <c r="D195" t="inlineStr">
         <is>
@@ -5480,7 +5480,7 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>52072</v>
+        <v>56046</v>
       </c>
       <c r="D203" t="inlineStr">
         <is>
@@ -6030,7 +6030,7 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>12999</v>
+        <v>13450</v>
       </c>
       <c r="D225" t="inlineStr">
         <is>
@@ -6130,7 +6130,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>93719</v>
+        <v>103999</v>
       </c>
       <c r="D229" t="inlineStr">
         <is>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>51860</v>
+        <v>51579</v>
       </c>
       <c r="D235" t="inlineStr">
         <is>
@@ -6605,7 +6605,7 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>168399</v>
+        <v>166199</v>
       </c>
       <c r="D248" t="inlineStr">
         <is>
@@ -7588,6 +7588,3881 @@
         </is>
       </c>
       <c r="E287" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>MLA859028844</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Estante Parrilla Rejilla Exhibidora Briket M4200 Original</t>
+        </is>
+      </c>
+      <c r="C288" t="n">
+        <v>33916</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/estante-parrilla-rejilla-exhibidora-briket-m4200-original/up/MLAU199682751?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=1&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA859028844&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>MLA1168637274</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Termostato Exhibidora Briket M1200/3200/4200/5000</t>
+        </is>
+      </c>
+      <c r="C289" t="n">
+        <v>26194</v>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/termostato-exhibidora-briket-m1200320042005000/up/MLAU154193232?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=2&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1168637274&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>MLA1455716959</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Estante Parrilla Rejilla Exhibidora Inelro Mt 12 14 17 X4 Un</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>123876</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/estante-parrilla-rejilla-exhibidora-inelro-mt-12-14-17-x4-un/up/MLAU2372569474?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=5&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1455716959&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>MLA1690765563</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Canasto Cajón Freezer Pozo Gafa Con Manijas Original X4 Unid</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>78038</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/canasto-cajon-freezer-pozo-gafa-con-manijas-original-x4-unid/up/MLAU2482216291?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=6&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1690765563&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>MLA1439285867</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Tapa Vidrio Curvo Freezer Inelro 550 Pi X1 Unidad Original</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>216197</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/tapa-vidrio-curvo-freezer-inelro-550-pi-x1-unidad-original/up/MLAU423240933?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=7&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1439285867&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>MLA2498568522</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Canasto Cajón Freezer Inelro Con Manijas Original X4 Unid Or</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>82406</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/canasto-cajon-freezer-inelro-con-manijas-original-x4-unid-or/up/MLAU3522833256?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=8&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA2498568522&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>MLA1969034292</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Parrilla Estante Heladera Exhibidora Inelro Mt-470 Original</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>31556</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/parrilla-estante-heladera-exhibidora-inelro-mt470-original/up/MLAU2877564080?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=9&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1969034292&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>MLA1568150357</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Canasto Cajón Freezer Briket Con Manijas Original X2 Unid Or</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
+        <v>41504</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/canasto-cajon-freezer-briket-con-manijas-original-x2-unid-or/up/MLAU3522831894?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=10&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1568150357&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>MLA1549147363</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Tapa Vidrio Curvo Freezer Frare Eh160 Vision Original</t>
+        </is>
+      </c>
+      <c r="C296" t="n">
+        <v>178154</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/tapa-vidrio-curvo-freezer-frare-eh160-vision-original/up/MLAU3451705931?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=11&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1549147363&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>MLA1121472343</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Manija Freezer Briket Todos Modelos Gastada Original</t>
+        </is>
+      </c>
+      <c r="C297" t="n">
+        <v>10819</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/manija-freezer-briket-todos-modelos-gastada-original/up/MLAU142384370?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=12&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1121472343&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>MLA2367085594</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Resorte Derecho Puerta Exhibidora Inelro Mt 980 Original</t>
+        </is>
+      </c>
+      <c r="C298" t="n">
+        <v>21125</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/resorte-derecho-puerta-exhibidora-inelro-mt-980-original/up/MLAU3423199957?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=13&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA2367085594&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>MLA3060244914</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Anaquel Acrílico Plano A Tornillo Heladera Bambi 1200 X3 Un</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
+        <v>70513</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/anaquel-acrilico-plano-a-tornillo-heladera-bambi-1200-x3-un/up/MLAU3840617647?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=14&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA3060244914&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>MLA859028841</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Termostato Heladera Briket Con Congelador Original</t>
+        </is>
+      </c>
+      <c r="C300" t="n">
+        <v>31937</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/termostato-heladera-briket-con-congelador-original/up/MLAU177004521?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=16&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA859028841&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>MLA1474494947</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Condensador Freezer Briket Fr3300 Refrigeración 60cm X 105cm</t>
+        </is>
+      </c>
+      <c r="C301" t="n">
+        <v>71394</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/condensador-freezer-briket-fr3300-refrigeracion-60cm-x-105cm/up/MLAU2995644572?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=17&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1474494947&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>MLA1691878051</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Kit Arranque Relay + Protector Termico Ptc Heladera 1/4hp</t>
+        </is>
+      </c>
+      <c r="C302" t="n">
+        <v>12834</v>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/kit-arranque-relay--protector-termico-ptc-heladera-14hp/up/MLAU3833139396?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=21&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1691878051&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>MLA3008562200</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Kit Arranque Relay + Protector Termico Ptc Heladera 1/5hp</t>
+        </is>
+      </c>
+      <c r="C303" t="n">
+        <v>10645</v>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/kit-arranque-relay--protector-termico-ptc-heladera-15hp/up/MLAU3829525230?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=22&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA3008562200&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>MLA2366953752</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Plastico Faldon Zocalo Para Exhibidora Inelro Bt 19 Original</t>
+        </is>
+      </c>
+      <c r="C304" t="n">
+        <v>67577</v>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plastico-faldon-zocalo-para-exhibidora-inelro-bt-19-original/up/MLAU3423130295?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=23&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA2366953752&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>MLA2045899802</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Burlete Exhibidora Briket Master M5000 68cm X 169cm Original</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>50903</v>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/burlete-exhibidora-briket-master-m5000-68cm-x-169cm-original/up/MLAU3112578262?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=24&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA2045899802&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>MLA1131886985</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Relay Rele Termico Ptc De 3 Y 4 Contactos Para Heladera</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
+        <v>7470</v>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/relay-rele-termico-ptc-de-3-y-4-contactos-para-heladera/up/MLAU146541088?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=27&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1131886985&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>MLA1957646540</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Parrilla Estante Bandeja Exhibidora Inelro Mt-750 Original</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>34711</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/parrilla-estante-bandeja-exhibidora-inelro-mt750-original/up/MLAU2747884813?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=28&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1957646540&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>MLA2046015170</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Burlete Exhibidora Inelro Mt 380 60,5cm X 141cm Original</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
+        <v>49359</v>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/burlete-exhibidora-inelro-mt-380-605cm-x-141cm-original/up/MLAU3112577206?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=29&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA2046015170&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>MLA931734340</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Plaqueta Potencia Electrolux Miriam</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>67716</v>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plaqueta-potencia-electrolux-miriam/up/MLAU204279793?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=30&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA931734340&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>MLA1965872136</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Tapa Vidrio Curvo Freezer Inelro 270 Pi X1 Unidad Original</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>119954</v>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/tapa-vidrio-curvo-freezer-inelro-270-pi-x1-unidad-original/up/MLAU2861249830?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=31&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1965872136&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>MLA1534264767</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Condensador Caracol 4 Vueltas Exhibidora Inelro Mt 11 Origin</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
+        <v>98319</v>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/condensador-caracol-4-vueltas-exhibidora-inelro-mt-11-origin/up/MLAU3425395794?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=32&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1534264767&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>MLA859028864</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Faldón Zócalo Exhibidora Briket Master 5000 M5000 Original</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
+        <v>36805</v>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/faldon-zocalo-exhibidora-briket-master-5000-m5000-original/up/MLAU177036853?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=35&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA859028864&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>MLA2374237654</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Resorte Izquierdo Puerta Exhibidora Inelro Mt 980 Original</t>
+        </is>
+      </c>
+      <c r="C313" t="n">
+        <v>21125</v>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/resorte-izquierdo-puerta-exhibidora-inelro-mt-980-original/up/MLAU3425251247?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=37&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA2374237654&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>MLA859028270</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Placa Evaporadora Heladera Briket 1610 1620 1810 Y Otras</t>
+        </is>
+      </c>
+      <c r="C314" t="n">
+        <v>77121</v>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/placa-evaporadora-heladera-briket-1610-1620-1810-y-otras/up/MLAU159037696?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=38&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA859028270&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>MLA1458300545</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Manijas Tapa Vidrio Freezer Briket Eh2500/3300/4500 X2 Unid</t>
+        </is>
+      </c>
+      <c r="C315" t="n">
+        <v>9007</v>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/manijas-tapa-vidrio-freezer-briket-eh250033004500-x2-unid/up/MLAU2664958505?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=39&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1458300545&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>MLA1696072999</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Parrilla Estante Heladera Exhibidora Inelro Mt 980 Color Neg</t>
+        </is>
+      </c>
+      <c r="C316" t="n">
+        <v>41239</v>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/parrilla-estante-heladera-exhibidora-inelro-mt-980-color-neg/up/MLAU3829892063?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=40&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1696072999&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>MLA1583456207</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Placa Evaporadora Heladera Universal 50cm X 50cm Cobre</t>
+        </is>
+      </c>
+      <c r="C317" t="n">
+        <v>111978</v>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/placa-evaporadora-heladera-universal-50cm-x-50cm-cobre/up/MLAU3559335907?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=41&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1583456207&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>MLA859028248</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Anaquel Acrílico Corto Heladera Bambi Briket 1610 1620 1630</t>
+        </is>
+      </c>
+      <c r="C318" t="n">
+        <v>8217</v>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/anaquel-acrilico-corto-heladera-bambi-briket-1610-1620-1630/up/MLAU197788859?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=43&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA859028248&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>MLA1415811199</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Anaquel Acrílico Botellas Heladera Briket 2100 1610 1810</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>11084</v>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/anaquel-acrilico-botellas-heladera-briket-2100-1610-1810/up/MLAU339050691?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=44&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1415811199&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>MLA2045886760</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Burlete Exhibidora Briket Master M1200 52cm X 75cm Original</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>32144</v>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/burlete-exhibidora-briket-master-m1200-52cm-x-75cm-original/up/MLAU3107184369?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=45&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA2045886760&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>MLA3060134764</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Tapa Vidrio Curvo Freezer Inelro Pi 350 Con Manija Original</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>200933</v>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/tapa-vidrio-curvo-freezer-inelro-pi-350-con-manija-original/up/MLAU3840486493?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=46&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA3060134764&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>MLA1458377969</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Manijas Tapa Vidrio Freezer Inelro Pi270/350/550 X2 Unidades</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>9896</v>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/manijas-tapa-vidrio-freezer-inelro-pi270350550-x2-unidades/up/MLAU2664959439?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=47&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1458377969&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>MLA1458274539</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Manijas Tapa Vidrio Curvo Freezer Frider Blanca X2 Unidades</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>9007</v>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/manijas-tapa-vidrio-curvo-freezer-frider-blanca-x2-unidades/up/MLAU2664955439?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=49&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA1458274539&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>MLA2989116560</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Liquido Limpia Evaporador Aire Acondicionado X 5 Litros</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>58602</v>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/liquido-limpia-evaporador-aire-acondicionado-x-5-litros/up/MLAU3816656319?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=50&amp;type=product&amp;tracking_id=b4bbe593-1588-4979-9eae-73f31cecfdd1&amp;wid=MLA2989116560&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>MLA1423369483</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Parrilla Estante Freezer Heladera Briket Modelo 1310/1410</t>
+        </is>
+      </c>
+      <c r="C325" t="n">
+        <v>26333</v>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/parrilla-estante-freezer-heladera-briket-modelo-13101410/up/MLAU362690545?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=3&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1423369483&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>MLA1438375482</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Cerradura Manija Freezer Briket Blanca Seguridad Traba Blanc</t>
+        </is>
+      </c>
+      <c r="C326" t="n">
+        <v>7711</v>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/cerradura-manija-freezer-briket-blanca-seguridad-traba-blanc/up/MLAU165086604?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=4&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1438375482&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>MLA1931247100</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Medio Estante Parrilla Bandeja Heladera Briket 1610/20/1810</t>
+        </is>
+      </c>
+      <c r="C327" t="n">
+        <v>21737</v>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/medio-estante-parrilla-bandeja-heladera-briket-1610201810/up/MLAU2127984373?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=6&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1931247100&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>MLA1535158333</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Plastico Faldon Zocalo Exhibidora Inelro Mt 12 14 17 Origina</t>
+        </is>
+      </c>
+      <c r="C328" t="n">
+        <v>33597</v>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plastico-faldon-zocalo-exhibidora-inelro-mt-12-14-17-origina/up/MLAU3427982828?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=7&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1535158333&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>MLA859028819</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Anaquel Acrílico Corto Bajo Heladera Bambi Briket 1610/20/3</t>
+        </is>
+      </c>
+      <c r="C329" t="n">
+        <v>9008</v>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/anaquel-acrilico-corto-bajo-heladera-bambi-briket-1610203/up/MLAU140072124?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=8&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA859028819&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>MLA1535107455</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Rejilla Plastica Lateral Cubremotor Freezer Inelro Original</t>
+        </is>
+      </c>
+      <c r="C330" t="n">
+        <v>16317</v>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/rejilla-plastica-lateral-cubremotor-freezer-inelro-original/up/MLAU3421449039?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=9&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1535107455&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>MLA2361165812</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Pala Plástica Forzador Inelro Original De 200mm Anti Horario</t>
+        </is>
+      </c>
+      <c r="C331" t="n">
+        <v>5953</v>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/pala-plastica-forzador-inelro-original-de-200mm-anti-horario/up/MLAU3420676319?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=10&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2361165812&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>MLA1472168955</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Puerta Heladera Exhibidora Inelro Mt 14 68cm X 142cm Orig</t>
+        </is>
+      </c>
+      <c r="C332" t="n">
+        <v>358729</v>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/puerta-heladera-exhibidora-inelro-mt-14-68cm-x-142cm-orig/up/MLAU2969586772?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=11&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1472168955&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>MLA1132407080</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Protector Termico Ptc Para Motor De 1/4 Hp</t>
+        </is>
+      </c>
+      <c r="C333" t="n">
+        <v>8060</v>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/protector-termico-ptc-para-motor-de-14-hp/up/MLAU145382787?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=12&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1132407080&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>MLA2989038682</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Agente Limpieza Cleaner Diluyente Industrial X 5 Litros Refr</t>
+        </is>
+      </c>
+      <c r="C334" t="n">
+        <v>41644</v>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/agente-limpieza-cleaner-diluyente-industrial-x-5-litros-refr/up/MLAU3826578892?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=13&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2989038682&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>MLA2366912530</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Tubo Led Plafon Touch 530mm Exhibidora Inelro Mt 300 400 470</t>
+        </is>
+      </c>
+      <c r="C335" t="n">
+        <v>130155</v>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/tubo-led-plafon-touch-530mm-exhibidora-inelro-mt-300-400-470/up/MLAU3429683174?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=14&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2366912530&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>59118</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Burlete Inferior Para Heladera Briket 1610 60,5cm X 109cm</t>
+        </is>
+      </c>
+      <c r="C336" t="n">
+        <v>42507</v>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>https://articulo.mercadolibre.com.ar/MLA-907774532-burlete-inferior-para-heladera-briket-1610-605cm-x-109cm-_JM?searchVariation=182080213853&amp;pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;searchVariation=182080213853&amp;search_layout=stack&amp;position=15&amp;type=item&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>MLA1487605725</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Burlete Exhibidora Briket M4200 M4300 64cm X 159cm Original</t>
+        </is>
+      </c>
+      <c r="C337" t="n">
+        <v>56425</v>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/burlete-exhibidora-briket-m4200-m4300-64cm-x-159cm-original/up/MLAU3112575306?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=16&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1487605725&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>MLA1607411813</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Panel Membrana Serigrafia Gafa / Electrolux Digifit Original</t>
+        </is>
+      </c>
+      <c r="C338" t="n">
+        <v>16500</v>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/panel-membrana-serigrafia-gafa--electrolux-digifit-original/up/MLAU3670477721?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=17&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1607411813&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>MLA1570863435</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Polea Lavarropas Drean Gold 1910 610 8.6 10.6 12.8 Original</t>
+        </is>
+      </c>
+      <c r="C339" t="n">
+        <v>56513</v>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/polea-lavarropas-drean-gold-1910-610-86-106-128-original/up/MLAU3523131219?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=18&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1570863435&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>MLA2686057358</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Plancha A Vapor Gardenia 2200w Con Rociador Color Rojo</t>
+        </is>
+      </c>
+      <c r="C340" t="n">
+        <v>51041</v>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plancha-a-vapor-gardenia-2200w-con-rociador-color-rojo/up/MLAU3679269611?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=19&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2686057358&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>MLA1535164873</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Placa Evaporadora Exhibidora Inelro Mt 120 Original</t>
+        </is>
+      </c>
+      <c r="C341" t="n">
+        <v>110119</v>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/placa-evaporadora-exhibidora-inelro-mt-120-original/up/MLAU3420974353?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=20&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1535164873&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>MLA1764201156</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Manija Tapa Vidrio Freezer Inelro Pi 270/350/550 X Unidad</t>
+        </is>
+      </c>
+      <c r="C342" t="n">
+        <v>4767</v>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/manija-tapa-vidrio-freezer-inelro-pi-270350550-x-unidad/up/MLAU369034404?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=21&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1764201156&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>MLA2361052780</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Pala Plástica Forzador Inelro Original De 230mm Anti Horario</t>
+        </is>
+      </c>
+      <c r="C343" t="n">
+        <v>5367</v>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/pala-plastica-forzador-inelro-original-de-230mm-anti-horario/up/MLAU3420811157?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=22&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2361052780&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>MLA1535182759</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Plastico Faldon Zocalo Curvo Exhibidora Inelro Mt 470 Origin</t>
+        </is>
+      </c>
+      <c r="C344" t="n">
+        <v>53639</v>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plastico-faldon-zocalo-curvo-exhibidora-inelro-mt-470-origin/up/MLAU3427879840?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=23&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1535182759&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>MLA2686723462</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Porta Sachet Heladera Electrolux Original Universal Gastado</t>
+        </is>
+      </c>
+      <c r="C345" t="n">
+        <v>15871</v>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/porta-sachet-heladera-electrolux-original-universal-gastado/up/MLAU3679666241?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=24&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2686723462&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>MLA2031288862</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Juego De Burletes Heladera Gafa Hgf 3880 300 380 58x110x59</t>
+        </is>
+      </c>
+      <c r="C346" t="n">
+        <v>64263</v>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/juego-de-burletes-heladera-gafa-hgf-3880-300-380-58x110x59/up/MLAU3067390125?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=25&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2031288862&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>MLA3008562202</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Kit Arranque Relay + Protector Termico Ptc Heladera 1/3hp</t>
+        </is>
+      </c>
+      <c r="C347" t="n">
+        <v>10645</v>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/kit-arranque-relay--protector-termico-ptc-heladera-13hp/up/MLAU3829526894?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=26&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA3008562202&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>MLA1368272463</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Aceite Para R134 / R404 X 1l Refrioil</t>
+        </is>
+      </c>
+      <c r="C348" t="n">
+        <v>28109</v>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/aceite-para-r134--r404-x-1l-refrioil/up/MLAU159181405?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=27&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1368272463&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>MLA1444403245</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Forzador Cuadrado 300mm 16w Exhibidora/freezer Refrigeración</t>
+        </is>
+      </c>
+      <c r="C349" t="n">
+        <v>36853</v>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/forzador-cuadrado-300mm-16w-exhibidorafreezer-refrigeracion/up/MLAU563469306?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=28&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1444403245&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>MLA1416826515</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Funda Cobertor De Limpieza Aire Acondicionado 2250 A 3000</t>
+        </is>
+      </c>
+      <c r="C350" t="n">
+        <v>36837</v>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/funda-cobertor-de-limpieza-aire-acondicionado-2250-a-3000/up/MLAU407654288?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=30&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1416826515&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>MLA2535849780</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Aro Balanceador Lavarropas Drean Concept 5.05 / C12 Original</t>
+        </is>
+      </c>
+      <c r="C351" t="n">
+        <v>46236</v>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/aro-balanceador-lavarropas-drean-concept-505--c12-original/up/MLAU3533995693?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=31&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2535849780&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>MLA1439461513</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Plaqueta (mc-l42) Flex Lavarropas Candy Gvsw286tc3</t>
+        </is>
+      </c>
+      <c r="C352" t="n">
+        <v>14723</v>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plaqueta-mcl42-flex-lavarropas-candy-gvsw286tc3/up/MLAU423718389?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=32&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1439461513&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>MLA1606303354</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Presostato Lavarropas Gafa Electronico Original 6500 7500</t>
+        </is>
+      </c>
+      <c r="C353" t="n">
+        <v>15690</v>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/presostato-lavarropas-gafa-electronico-original-6500-7500/up/MLAU167063133?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=33&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1606303354&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>MLA2604393810</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Control Remoto Aire Acondicionado Hitachi  R5m/e Original</t>
+        </is>
+      </c>
+      <c r="C354" t="n">
+        <v>11408</v>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/control-remoto-aire-acondicionado-hitachi--r5me-original/up/MLAU3635582476?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=34&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2604393810&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>MLA2686053400</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Anaquel Frascos Gafa Superior 47 X 7 Original Gastado</t>
+        </is>
+      </c>
+      <c r="C355" t="n">
+        <v>16875</v>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/anaquel-frascos-gafa-superior-47-x-7-original-gastado/up/MLAU3679642055?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=35&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2686053400&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>MLA2686067086</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Bandeja Desagote Motor Electrolux Gafa Gastado Original</t>
+        </is>
+      </c>
+      <c r="C356" t="n">
+        <v>8466</v>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/bandeja-desagote-motor-electrolux-gafa-gastado-original/up/MLAU3679664691?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=36&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2686067086&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>MLA1574638857</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Mirilla Visor Puerta Acrilico Lavarropas Drean Excellent Or</t>
+        </is>
+      </c>
+      <c r="C357" t="n">
+        <v>56218</v>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/mirilla-visor-puerta-acrilico-lavarropas-drean-excellent-or/up/MLAU3541181160?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=37&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1574638857&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>MLA1171030381</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Frente Panel Drean Concept 5.05 V1 Sin Visor</t>
+        </is>
+      </c>
+      <c r="C358" t="n">
+        <v>63822</v>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/frente-panel-drean-concept-505-v1-sin-visor/up/MLAU154239122?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=38&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1171030381&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>MLA2686093042</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Anaquel Acrilico Chico Heladera Electrolux 22 X 10 Original</t>
+        </is>
+      </c>
+      <c r="C359" t="n">
+        <v>15268</v>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/anaquel-acrilico-chico-heladera-electrolux-22-x-10-original/up/MLAU3687994698?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=39&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2686093042&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>MLA1775529830</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Embrague Lavarropas Buje De Arrastre Drean Concept 5.05</t>
+        </is>
+      </c>
+      <c r="C360" t="n">
+        <v>6666</v>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/embrague-lavarropas-buje-de-arrastre-drean-concept-505/up/MLAU373506266?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=40&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1775529830&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>MLA931726733</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Plaqueta Interfase Electrolux Miriam Fuzzy Wash Con Visor</t>
+        </is>
+      </c>
+      <c r="C361" t="n">
+        <v>41556</v>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plaqueta-interfase-electrolux-miriam-fuzzy-wash-con-visor/up/MLAU203975071?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=41&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA931726733&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>MLA1422484517</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Plaqueta Interface Electrolux Digital Wash Sin Visor Origin</t>
+        </is>
+      </c>
+      <c r="C362" t="n">
+        <v>38373</v>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plaqueta-interface-electrolux-digital-wash-sin-visor-origin/up/MLAU360242794?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=42&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1422484517&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>MLA2357170678</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Tira Lampara Led Freezer Inelro Fih 350 Pi Plus 94cm Origin</t>
+        </is>
+      </c>
+      <c r="C363" t="n">
+        <v>91412</v>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/tira-lampara-led-freezer-inelro-fih-350-pi-plus-94cm-origin/up/MLAU3425902920?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=43&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2357170678&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>MLA1835784306</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Plaqueta (mc-l42) Flex Lavarropas Longvie L16508/l16510</t>
+        </is>
+      </c>
+      <c r="C364" t="n">
+        <v>17596</v>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plaqueta-mcl42-flex-lavarropas-longvie-l16508l16510/up/MLAU400029220?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=44&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1835784306&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>MLA1980250616</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Caja Mecanismo Lavarropas Gafa 6000 6100 6500 7000 7500</t>
+        </is>
+      </c>
+      <c r="C365" t="n">
+        <v>92223</v>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/caja-mecanismo-lavarropas-gafa-6000-6100-6500-7000-7500/up/MLAU2901503831?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=45&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1980250616&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>MLA1708309070</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Plaqueta (mc-l41) Flex Lavarropas Gvs128/214 Gvf141 Candy</t>
+        </is>
+      </c>
+      <c r="C366" t="n">
+        <v>18613</v>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plaqueta-mcl41-flex-lavarropas-gvs128214-gvf141-candy/up/MLAU338978473?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=46&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA1708309070&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>MLA2357273284</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Tira Lampara Led Freezer Inelro Fih 270 Pi Plus 73.5cm Orig</t>
+        </is>
+      </c>
+      <c r="C367" t="n">
+        <v>82652</v>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/tira-lampara-led-freezer-inelro-fih-270-pi-plus-735cm-orig/up/MLAU3419225317?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=47&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA2357273284&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>37383</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Burlete Inferior Para Heladera Briket 1600/1610/1620/1630</t>
+        </is>
+      </c>
+      <c r="C368" t="n">
+        <v>42507</v>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>https://articulo.mercadolibre.com.ar/MLA-1399971555-burlete-inferior-para-heladera-briket-1600161016201630-_JM?searchVariation=179519255668&amp;pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;searchVariation=179519255668&amp;search_layout=stack&amp;position=48&amp;type=item&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>MLA923952070</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Plaqueta Drean Concept Fuzzy Logic Tech Con Visor</t>
+        </is>
+      </c>
+      <c r="C369" t="n">
+        <v>71045</v>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plaqueta-drean-concept-fuzzy-logic-tech-con-visor/up/MLAU196890636?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=49&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA923952070&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>MLA859027478</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Termostato Para Freezer Dual Briket</t>
+        </is>
+      </c>
+      <c r="C370" t="n">
+        <v>27864</v>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/termostato-para-freezer-dual-briket/up/MLAU139268035?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=50&amp;type=product&amp;tracking_id=bba0c71e-cd97-4346-9261-811ef24452bd&amp;wid=MLA859027478&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>MLA1473340057</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Bisagra Sin Resorte Freezer Pozo Bambi Original</t>
+        </is>
+      </c>
+      <c r="C371" t="n">
+        <v>17423</v>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/bisagra-sin-resorte-freezer-pozo-bambi-original/up/MLAU2978545333?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=3&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1473340057&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>MLA1689449143</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Interruptor Luz Forzador Heladera Exhibidora Briket Original</t>
+        </is>
+      </c>
+      <c r="C372" t="n">
+        <v>13405</v>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/interruptor-luz-forzador-heladera-exhibidora-briket-original/up/MLAU3828827348?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=4&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1689449143&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>MLA1706342077</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Estante Parrilla Exhibidora Heladera Inelro Mt 12 14 17 X2</t>
+        </is>
+      </c>
+      <c r="C373" t="n">
+        <v>71474</v>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/estante-parrilla-exhibidora-heladera-inelro-mt-12-14-17-x2/up/MLAU3840192667?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=5&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1706342077&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>MLA3065277876</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Manijas Tapa Vidrio Freezer Inelro Pi270/350/550 X10 Unid</t>
+        </is>
+      </c>
+      <c r="C374" t="n">
+        <v>32301</v>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/manijas-tapa-vidrio-freezer-inelro-pi270350550-x10-unid/up/MLAU3842000999?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=6&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA3065277876&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>MLA1122584853</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Eje Soporte Drean Excellent 166 Punta Redonda 03 / 03</t>
+        </is>
+      </c>
+      <c r="C375" t="n">
+        <v>24136</v>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/eje-soporte-drean-excellent-166-punta-redonda-03--03/up/MLAU143171482?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=7&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1122584853&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>MLA1707958439</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Manijas Tapa Vidrio Freezer Inelro Pi270/350/550 X6 Unidades</t>
+        </is>
+      </c>
+      <c r="C376" t="n">
+        <v>20840</v>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/manijas-tapa-vidrio-freezer-inelro-pi270350550-x6-unidades/up/MLAU3841982305?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=8&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1707958439&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>MLA1397767747</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Varilla De Plata Negra Tipo Harris X 15unidades</t>
+        </is>
+      </c>
+      <c r="C377" t="n">
+        <v>34240</v>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/varilla-de-plata-negra-tipo-harris-x-15unidades/up/MLAU178713891?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=9&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1397767747&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>MLA1706314801</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Anaquel Acrílico Plano Heladera Bambi 1200 / 1600 A Tornillo</t>
+        </is>
+      </c>
+      <c r="C378" t="n">
+        <v>23504</v>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/anaquel-acrilico-plano-heladera-bambi-1200--1600-a-tornillo/up/MLAU3850346130?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=10&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1706314801&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>MLA1687673225</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Liquido Limpia Condensador Radiador Desincrustrante X1 Litro</t>
+        </is>
+      </c>
+      <c r="C379" t="n">
+        <v>12989</v>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/liquido-limpia-condensador-radiador-desincrustrante-x1-litro/up/MLAU3826578976?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=11&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1687673225&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>MLA2989142118</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Agente Limpieza Cleaner Diluyente Industrial X 1 Litro Refri</t>
+        </is>
+      </c>
+      <c r="C380" t="n">
+        <v>10779</v>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/agente-limpieza-cleaner-diluyente-industrial-x-1-litro-refri/up/MLAU3826577652?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=12&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA2989142118&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>MLA1612937949</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Puerta Heladera Exhibidora Inelro Mt 12 67,5 X 120 Cm Origin</t>
+        </is>
+      </c>
+      <c r="C381" t="n">
+        <v>321040</v>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/puerta-heladera-exhibidora-inelro-mt-12-675-x-120-cm-origin/up/MLAU3690728084?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=13&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1612937949&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>MLA1685005931</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Corta Caño Tubo Cobre Y Aluminio Refrigeracion 3/16 A 3/4</t>
+        </is>
+      </c>
+      <c r="C382" t="n">
+        <v>19137</v>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/corta-cano-tubo-cobre-y-aluminio-refrigeracion-316-a-34/up/MLAU3820561924?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=14&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1685005931&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>MLA3065123610</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Manijas Tapa Vidrio Freezer Inelro 270/350/550 Pi Plus X6 Un</t>
+        </is>
+      </c>
+      <c r="C383" t="n">
+        <v>31243</v>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/manijas-tapa-vidrio-freezer-inelro-270350550-pi-plus-x6-un/up/MLAU3841960127?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=15&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA3065123610&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>MLA1612899409</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Puerta Exhibidora Inelro Mt 12 67,5 X 120 Original Verde</t>
+        </is>
+      </c>
+      <c r="C384" t="n">
+        <v>307204</v>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/puerta-exhibidora-inelro-mt-12-675-x-120-original-verde/up/MLAU3690730004?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=16&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1612899409&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>MLA2989013128</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Liquido Detector De Fugas Exterior Refrigeracion X 1/2 Litro</t>
+        </is>
+      </c>
+      <c r="C385" t="n">
+        <v>19154</v>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/liquido-detector-de-fugas-exterior-refrigeracion-x-12-litro/up/MLAU3826577658?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=17&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA2989013128&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>MLA2989077698</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Aceite Motocompresor R410 / R407 X 1 Litro Refrigeracion</t>
+        </is>
+      </c>
+      <c r="C386" t="n">
+        <v>22886</v>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/aceite-motocompresor-r410--r407-x-1-litro-refrigeracion/up/MLAU3826577650?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=18&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA2989077698&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>MLA3064152046</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Estante Parrilla Rejilla Exhibidora Inelro Mt 19 X4 Un Orig</t>
+        </is>
+      </c>
+      <c r="C387" t="n">
+        <v>144446</v>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/estante-parrilla-rejilla-exhibidora-inelro-mt-19-x4-un-orig/up/MLAU3841637807?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=19&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA3064152046&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>MLA1706573345</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Estante Parrilla Rejilla Exhibidora Inelro Mt 19 X2 Un Orig</t>
+        </is>
+      </c>
+      <c r="C388" t="n">
+        <v>71201</v>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/estante-parrilla-rejilla-exhibidora-inelro-mt-19-x2-un-orig/up/MLAU3850985702?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=20&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1706573345&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>MLA2989142116</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Aceite Motocompresor R12 / R22 X 1 Litro Refrioil Refrigerac</t>
+        </is>
+      </c>
+      <c r="C389" t="n">
+        <v>14226</v>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/aceite-motocompresor-r12--r22-x-1-litro-refrioil-refrigerac/up/MLAU3826577654?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=21&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA2989142116&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>MLA3059312490</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Estante Acrílico Bandeja Heladera Gafa Eurosystem X2 Origina</t>
+        </is>
+      </c>
+      <c r="C390" t="n">
+        <v>57239</v>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/estante-acrilico-bandeja-heladera-gafa-eurosystem-x2-origina/up/MLAU3840009207?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=22&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA3059312490&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>MLA2002465420</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Bisagra Sin Resorte Freezer Pozo Bambi Original X2 Unidades</t>
+        </is>
+      </c>
+      <c r="C391" t="n">
+        <v>31813</v>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/bisagra-sin-resorte-freezer-pozo-bambi-original-x2-unidades/up/MLAU2978546851?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=23&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA2002465420&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>MLA1157342227</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Termostato Ambiente Heladera Comercial +- 35°c Refrigeracion</t>
+        </is>
+      </c>
+      <c r="C392" t="n">
+        <v>14191</v>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/termostato-ambiente-heladera-comercial--35c-refrigeracion/up/MLAU152515479?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=24&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1157342227&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>MLA2988999792</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Aceite Motocompresor R134 X 1/2 Litro Refrioil Refrigeracion</t>
+        </is>
+      </c>
+      <c r="C393" t="n">
+        <v>16054</v>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/aceite-motocompresor-r134-x-12-litro-refrioil-refrigeracion/up/MLAU3826577656?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=25&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA2988999792&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>MLA2900514784</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Taladro Percutor Impacto Daewoo 3300rpm 750w Naranja 50hz</t>
+        </is>
+      </c>
+      <c r="C394" t="n">
+        <v>97332</v>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/taladro-percutor-impacto-daewoo-3300rpm-750w-naranja-50hz/up/MLAU3803752071?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=26&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA2900514784&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>MLA3068718030</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Tapa Vidrio Curvo Freezer Inelro Pi 550 Con Manija Original</t>
+        </is>
+      </c>
+      <c r="C395" t="n">
+        <v>204358</v>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/tapa-vidrio-curvo-freezer-inelro-pi-550-con-manija-original/up/MLAU3854566708?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=27&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA3068718030&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>MLA1600761000</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Robinete 5/8 Curvo R22 Refrigeracion</t>
+        </is>
+      </c>
+      <c r="C396" t="n">
+        <v>36009</v>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/robinete-58-curvo-r22-refrigeracion/up/MLAU168003212?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=28&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1600761000&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>MLA1419698641</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Valvula Inversora Aire Condicionado 3/8-1/2 R410</t>
+        </is>
+      </c>
+      <c r="C397" t="n">
+        <v>62211</v>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/valvula-inversora-aire-condicionado-3812-r410/up/MLAU351968333?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=29&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1419698641&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>MLA1445229647</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Llave Crique Refrigeración 3/16 1/4 1/2 9/16 Ct-123 Criket</t>
+        </is>
+      </c>
+      <c r="C398" t="n">
+        <v>11306</v>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/llave-crique-refrigeracion-316-14-12-916-ct123-criket/up/MLAU633288332?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=30&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1445229647&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>MLA1612950895</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Puerta Exhibidora Inelro Mt 17 68 X 163cm Original Verde</t>
+        </is>
+      </c>
+      <c r="C399" t="n">
+        <v>365758</v>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/puerta-exhibidora-inelro-mt-17-68-x-163cm-original-verde/up/MLAU3690730006?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=31&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1612950895&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>MLA2362785344</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Plastico Faldon Zocalo Exhibidora Inelro Mt 12 14 17 Negro O</t>
+        </is>
+      </c>
+      <c r="C400" t="n">
+        <v>32754</v>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plastico-faldon-zocalo-exhibidora-inelro-mt-12-14-17-negro-o/up/MLAU3421376045?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=32&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA2362785344&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>MLA2989013136</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Liquido Limpia Filtros Aire Acondicionado Desengrasante</t>
+        </is>
+      </c>
+      <c r="C401" t="n">
+        <v>13502</v>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/liquido-limpia-filtros-aire-acondicionado-desengrasante/up/MLAU3816655331?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=33&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA2989013136&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>MLA1687686235</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Liquido Limpia Evaporador Aire Acondicionado X 1 Litro Refri</t>
+        </is>
+      </c>
+      <c r="C402" t="n">
+        <v>12447</v>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/liquido-limpia-evaporador-aire-acondicionado-x-1-litro-refri/up/MLAU3816655251?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=34&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1687686235&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>MLA1372358139</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Plaqueta (mc-l40) Flex Lavarropas Cvst810t/ Ls18012 Candy</t>
+        </is>
+      </c>
+      <c r="C403" t="n">
+        <v>18006</v>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/plaqueta-mcl40-flex-lavarropas-cvst810t-ls18012-candy/up/MLAU159568035?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=35&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1372358139&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>MLA1445538901</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Puerta Heladera Exhibidora Vertical Briket Master 5000 M5000</t>
+        </is>
+      </c>
+      <c r="C404" t="n">
+        <v>405670</v>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/puerta-heladera-exhibidora-vertical-briket-master-5000-m5000/up/MLAU652350753?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=36&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA1445538901&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>MLA2367055818</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Tubo Led Plafon Touch 630mm Exhibidora Inelro Mt 19 Original</t>
+        </is>
+      </c>
+      <c r="C405" t="n">
+        <v>144175</v>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/tubo-led-plafon-touch-630mm-exhibidora-inelro-mt-19-original/up/MLAU3423073569?pdp_filters=official_store%3A141122#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=37&amp;type=product&amp;tracking_id=8035a304-168b-4905-9ef0-7861c75350fd&amp;wid=MLA2367055818&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Segui group</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>MLA2034207928</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Juego Bujias Cocina Orbis Convecta Sourdillon Originales</t>
+        </is>
+      </c>
+      <c r="C406" t="n">
+        <v>85460</v>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.ar/mclics/clicks/external/MLA/count?a=QjTx1c8iSqy8%2Bc76YgJV3TlTuE0l5Vh9yK0lboavrSyVEs8yrDClFy5c75I0DMBNscpxNuhUka0vI9PoCAzhMw4uSp3l9E4KKBTc8Y8DbhpziisdAeVrS4gZmxO2g3W6GBSHANZFZQ5gl9ldPrlZSqkibs7IhwY37pf931WV%2BU9kGs7JITVtqgpb1gfIjtw%2B6jGJm%2FV9WX270uR%2BCM39RSY%2BZBUcNldY32z6%2BIi4FbiOOjdTmSgmgd%2FpRUYlVqtZabt7RvZ2zZiN2Sl7XJEdDfncpU7zIxLhjfAcbd6%2BmNFpBZbOm5atDDr13XhDxHE3z1x3NCdpW0aCEFJbShU2whd%2B8%2BcGiwSLltRarRN1ebwotIbfiavG8Jjo5fjGVOYOIZyZdn%2FTNTKTftL5PXH6HGlkPNuFmpMAnB1i2Mf7P92sOcYdM1Y22nOhbk9c%2FTDRRA0UwiVBkfUs0W%2B88mnQ4jIj2pQ9fVQ8duJwmk%2FEUZNabYC4%2BrpRyZa3iDaNsUE7Q94VJ1YUvzvbt5mCiay8ky1gt2zP3xof01HJ2zDX7IeNi3qSVpN7MV1Kp6uZkObO3YXKs2YzDfPzsTpjfphuSWcs5VI6bsxxYnolxc2pTsgV3pIkf3sXfq54Z30AoSzxnh08IChGPdNDQxxkzrK7uKMIvQNIIv24firqmx%2FXIhihb3Ski7BaUs%2BOkTqDFhNE%2FNq9X3M%2BKCNhEnxKnAek2OPErW4%2B2ZdweVtpFTQuKpY4W3OSYKsx5Cm9RTiNyA6wBafO2V18760%2FRfUftbLULqPsfrM4qGL0OZxvByLTKEw7RY5tEeqskLg2eUxGz%2FLsPWntIcN16p0mxQ5wB7%2BTqppoo6lccO83E5Dwayn0BduyOw6fmSqtpU7TyW5B34dnPDOh%2Bk0p%2BYKQl%2BfFjTNqCpYL2MYnIl0SekG%2FvhkAy3defz%2BXyz1XW5jgEYze8TpRUAnHXN2CkZQ3pba0Ps5K5qIo%2BhugKFGvrYVLcWVMsbAjDA%2FriuWGAqI%3D&amp;pdp_filters=item_id%3AMLA2034207928#polycard_client=search-web-mobile&amp;is_advertising=true&amp;searchVariation=MLAU3076177161&amp;backend_model=search-backend&amp;be_origin=backend&amp;search_layout=stack&amp;position=1&amp;type=pad&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA2034207928&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>MLA733632715</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Camara De Agua Orbis Tonka Repuesto Nuevo</t>
+        </is>
+      </c>
+      <c r="C407" t="n">
+        <v>92920</v>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/camara-de-agua-orbis-tonka-repuesto-nuevo/up/MLAU191182199#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=3&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA733632715&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>MLA1119855577</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Optica Orion 1996 Izquierda</t>
+        </is>
+      </c>
+      <c r="C408" t="n">
+        <v>117427</v>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/optica-orion-1996-izquierda/up/MLAU145602372#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=4&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA1119855577&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>51630</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Optica Chevrolet Monza 1991 92 93 94 95 95 96 1997</t>
+        </is>
+      </c>
+      <c r="C409" t="n">
+        <v>181977</v>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>https://articulo.mercadolibre.com.ar/MLA-2050416982-optica-chevrolet-monza-1991-92-93-94-95-95-96-1997-_JM?searchVariation=183339697434#polycard_client=search-web-mobile&amp;be_origin=backend&amp;searchVariation=183339697434&amp;search_layout=stack&amp;position=6&amp;type=item&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>MLA712909740</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Varios Repuestos Consultas</t>
+        </is>
+      </c>
+      <c r="C410" t="n">
+        <v>80800</v>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/varios-repuestos-consultas/up/MLAU269084584#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=12&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA712909740&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>MLA63806450</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Curso De Manga 05 (incluye Portaminas Verde Con Minas 07 Hb De Repuesto), De Sin Autor. Editorial Fasciculos Coleccionables (ff)</t>
+        </is>
+      </c>
+      <c r="C411" t="n">
+        <v>14170</v>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/curso-de-manga-05-incluye-portaminas-verde-con-minas-07-hb-de-repuesto-de-sin-autor-editorial-fasciculos-coleccionables-ff/p/MLA63806450#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=15&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA2737902212&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>MLA923020656</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Catalogo De Repuestos Vw Gol G1</t>
+        </is>
+      </c>
+      <c r="C412" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/catalogo-de-repuestos-vw-gol-g1/up/MLAU199520449#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=18&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA923020656&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>MLA2434803678</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Qué Es La Propiedad? - Pierre Joseph Proudhon - Orbis</t>
+        </is>
+      </c>
+      <c r="C413" t="n">
+        <v>6450</v>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/que-es-la-propiedad--pierre-joseph-proudhon--orbis/up/MLAU3487402450#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=20&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA2434803678&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>44585</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Agenda 2025 Citanova Leo Carpeta Cuero Vaca Premium 14 X18,5</t>
+        </is>
+      </c>
+      <c r="C414" t="n">
+        <v>271650</v>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>https://articulo.mercadolibre.com.ar/MLA-1908348580-agenda-2025-citanova-leo-carpeta-cuero-vaca-premium-14-x185-_JM?searchVariation=184841474213#polycard_client=search-web-mobile&amp;be_origin=backend&amp;searchVariation=184841474213&amp;search_layout=stack&amp;position=24&amp;type=item&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>MLA1478440583</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Burlete Enterizo Mod. Anterior Orbis Convecta Donna Ragazza</t>
+        </is>
+      </c>
+      <c r="C415" t="n">
+        <v>48348</v>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/burlete-enterizo-mod-anterior-orbis-convecta-donna-ragazza/up/MLAU3030448129#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=25&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA1478440583&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>MLA1501686237</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Aros Pet-bioesferas/autolimpiantes P/biodigestor 4cm X100u</t>
+        </is>
+      </c>
+      <c r="C416" t="n">
+        <v>24999</v>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/aros-petbioesferasautolimpiantes-pbiodigestor-4cm-x100u/up/MLAU3215073718#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=28&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA1501686237&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>MLA2573500194</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Municiones  Balas Repuesto X 20000 Unidades Hidrogel Blaster</t>
+        </is>
+      </c>
+      <c r="C417" t="n">
+        <v>9600</v>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/municiones--balas-repuesto-x-20000-unidades-hidrogel-blaster/up/MLAU3568926828#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=29&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA2573500194&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>MLA680718198</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Circuito Impreso Trasero Izquierdo Ford Orion Original Arteb</t>
+        </is>
+      </c>
+      <c r="C418" t="n">
+        <v>165000</v>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/circuito-impreso-trasero-izquierdo-ford-orion-original-arteb/up/MLAU363923986#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=33&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA680718198&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>MLA1435443343</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Ficha Alternador Y Bulbo Aceite Volkswagen 1 Via</t>
+        </is>
+      </c>
+      <c r="C419" t="n">
+        <v>3360</v>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/ficha-alternador-y-bulbo-aceite-volkswagen-1-via/up/MLAU395427423#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=36&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA1435443343&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>MLA1169376528</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Termostato Termo Eléctrico Digital Orbis 50/80 Litros Eo/no</t>
+        </is>
+      </c>
+      <c r="C420" t="n">
+        <v>356264</v>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/termostato-termo-electrico-digital-orbis-5080-litros-eono/up/MLAU228609168#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=37&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA1169376528&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>22793</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Repuesto Cuaderno Inteligente, Planner Mensual A5 - 120gr.</t>
+        </is>
+      </c>
+      <c r="C421" t="n">
+        <v>8100</v>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>https://articulo.mercadolibre.com.ar/MLA-2039850388-repuesto-cuaderno-inteligente-planner-mensual-a5-120gr-_JM?searchVariation=185448429072#polycard_client=search-web-mobile&amp;be_origin=backend&amp;searchVariation=185448429072&amp;search_layout=stack&amp;position=38&amp;type=item&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>MLA1488677625</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Juego Opticas Chevrolet Monza 1991 92 93 94 95 95 96 1997</t>
+        </is>
+      </c>
+      <c r="C422" t="n">
+        <v>352294</v>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/juego-opticas-chevrolet-monza-1991-92-93-94-95-95-96-1997/up/MLAU3116975539#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=40&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA1488677625&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>MLA724295874</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Manual De Repuestos Tractor John Deere 730</t>
+        </is>
+      </c>
+      <c r="C423" t="n">
+        <v>70426</v>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/manual-de-repuestos-tractor-john-deere-730/up/MLAU270987242#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=42&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA724295874&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>MLA1556259969</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Estudios Sobre La Histeria Y Otros Ensayos - Freud - Orbis</t>
+        </is>
+      </c>
+      <c r="C424" t="n">
+        <v>4770</v>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/estudios-sobre-la-histeria-y-otros-ensayos--freud--orbis/up/MLAU3482084543#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=44&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA1556259969&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>MLA1557189179</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Critica De La Teoria Del Desarrollo- Bauer- Orbis</t>
+        </is>
+      </c>
+      <c r="C425" t="n">
+        <v>6990</v>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/critica-de-la-teoria-del-desarrollo-bauer-orbis/up/MLAU3483840297#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=45&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA1557189179&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>MLA1555979537</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Mandingo - Kyle Onstott - Orbis</t>
+        </is>
+      </c>
+      <c r="C426" t="n">
+        <v>5940</v>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/mandingo--kyle-onstott--orbis/up/MLAU3480522115#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=49&amp;type=product&amp;tracking_id=93bbd61a-10f6-4ff8-aefa-7a5151321580&amp;wid=MLA1555979537&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>MLA729423665</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Manual De Repuestos Tractor Deutz A70 Caja 4ta</t>
+        </is>
+      </c>
+      <c r="C427" t="n">
+        <v>65426</v>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/manual-de-repuestos-tractor-deutz-a70-caja-4ta/up/MLAU271331442#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=5&amp;type=product&amp;tracking_id=6645e5cf-b8cd-4863-a0e3-8322d92062d7&amp;wid=MLA729423665&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>MLA2038158510</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Mantenimiento Del Soporte De Agarre Del Mango Frontal Del La</t>
+        </is>
+      </c>
+      <c r="C428" t="n">
+        <v>18847</v>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/drill-side-front-handle-adjustment-59-65mm-grip-support-pp/p/MLA2038158510#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=12&amp;type=product&amp;tracking_id=6645e5cf-b8cd-4863-a0e3-8322d92062d7&amp;wid=MLA3126465730&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>MLA2389662394</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>John Fowles La Mujer Del Teniente Frances 1 Y 2 Orbis T Dura</t>
+        </is>
+      </c>
+      <c r="C429" t="n">
+        <v>14900</v>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/john-fowles-la-mujer-del-teniente-frances-1-y-2-orbis-t-dura/up/MLAU3444422536#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=15&amp;type=product&amp;tracking_id=6645e5cf-b8cd-4863-a0e3-8322d92062d7&amp;wid=MLA2389662394&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>MLA1542974627</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Jacqueline Sussan. El Valle De Las Muñecas Orbis Tapa Dura</t>
+        </is>
+      </c>
+      <c r="C430" t="n">
+        <v>14900</v>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/jacqueline-sussan-el-valle-de-las-munecas-orbis-tapa-dura/up/MLAU3439118879#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=18&amp;type=product&amp;tracking_id=6645e5cf-b8cd-4863-a0e3-8322d92062d7&amp;wid=MLA1542974627&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>MLA2023383715</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Álbum En P De 128 Bolsillos De Repuesto Para Películas Insta</t>
+        </is>
+      </c>
+      <c r="C431" t="n">
+        <v>17569</v>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/128-pockets-p-album-book-replacement-for-films-instant/p/MLA2023383715#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=19&amp;type=product&amp;tracking_id=6645e5cf-b8cd-4863-a0e3-8322d92062d7&amp;wid=MLA1533966193&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>MLA2622346450</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Distribuidor Orion Pointer 1.6 Inyeccion Bosch 9230087224</t>
+        </is>
+      </c>
+      <c r="C432" t="n">
+        <v>140000</v>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/distribuidor-orion-pointer-16-inyeccion-bosch-9230087224/up/MLAU3651565292#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=27&amp;type=product&amp;tracking_id=6645e5cf-b8cd-4863-a0e3-8322d92062d7&amp;wid=MLA2622346450&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>50289</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Cartas De Adivinación: Oráculos - Tarot - Aguilar</t>
+        </is>
+      </c>
+      <c r="C433" t="n">
+        <v>62900</v>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>https://articulo.mercadolibre.com.ar/MLA-865425705-cartas-de-adivinacion-oraculos-tarot-aguilar-_JM?searchVariation=59065533943#polycard_client=search-web-mobile&amp;be_origin=backend&amp;searchVariation=59065533943&amp;search_layout=stack&amp;position=28&amp;type=item&amp;tracking_id=6645e5cf-b8cd-4863-a0e3-8322d92062d7</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>MLA30711911</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Introducing Theologies Of Religion, De Paul F. Knitter. Editorial Orbis Books (usa), Tapa Blanda En Inglés</t>
+        </is>
+      </c>
+      <c r="C434" t="n">
+        <v>115799</v>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/introducing-theologies-of-religion-de-paul-f-knitter-editorial-orbis-books-usa-tapa-blanda-en-ingles/p/MLA30711911#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=42&amp;type=product&amp;tracking_id=6645e5cf-b8cd-4863-a0e3-8322d92062d7&amp;wid=MLA2305340328&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>MLA1480648283</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Orbis Ultra: El Vínculo Entre Mundos</t>
+        </is>
+      </c>
+      <c r="C435" t="n">
+        <v>130466</v>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/orbis-ultra-el-vinculo-entre-mundos/up/MLAU3050053001#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=5&amp;type=product&amp;tracking_id=2e8365dc-0eb4-4a06-b376-8750fa5af709&amp;wid=MLA1480648283&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>MLA1758666949</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Calefón A Gas Orbis 14 Litros Como Repuesto</t>
+        </is>
+      </c>
+      <c r="C436" t="n">
+        <v>249900</v>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/calefon-a-gas-orbis-14-litros-como-repuesto/up/MLAU3908379431#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=34&amp;type=product&amp;tracking_id=2e8365dc-0eb4-4a06-b376-8750fa5af709&amp;wid=MLA1758666949&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>MLA3210533828</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Calefon Orbis 20l 320kso, P/reparar O Repuestos</t>
+        </is>
+      </c>
+      <c r="C437" t="n">
+        <v>380000</v>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/calefon-orbis-20l-320kso-preparar-o-repuestos/up/MLAU3904739003#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=36&amp;type=product&amp;tracking_id=2e8365dc-0eb4-4a06-b376-8750fa5af709&amp;wid=MLA3210533828&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>MLA2863038464</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Botonera De Calefon Orbis. Reparada .tengo Otros Repuestos</t>
+        </is>
+      </c>
+      <c r="C438" t="n">
+        <v>130000</v>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/botonera-de-calefon-orbis-reparada-tengo-otros-repuestos/up/MLAU3798217234#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=37&amp;type=product&amp;tracking_id=2e8365dc-0eb4-4a06-b376-8750fa5af709&amp;wid=MLA2863038464&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>MLA1617622085</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>El Banquete / Fedón / Fedro - Platon - Ed: Orbis</t>
+        </is>
+      </c>
+      <c r="C439" t="n">
+        <v>17500</v>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/el-banquete--fedon--fedro--platon--ed-orbis/up/MLAU3689907513#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=40&amp;type=product&amp;tracking_id=2e8365dc-0eb4-4a06-b376-8750fa5af709&amp;wid=MLA1617622085&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>MLA2032358526</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Obras Selectas George Simenon, Editorial Orbis. Tapa Dura.</t>
+        </is>
+      </c>
+      <c r="C440" t="n">
+        <v>8250</v>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/obras-selectas-george-simenon-editorial-orbis-tapa-dura/up/MLAU3075660642#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=41&amp;type=product&amp;tracking_id=2e8365dc-0eb4-4a06-b376-8750fa5af709&amp;wid=MLA2032358526&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>MLA1470455752</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Colección Hyspamerica Orbis - Ver Títulos En Descripcion</t>
+        </is>
+      </c>
+      <c r="C441" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/coleccion-hyspamerica-orbis--ver-titulos-en-descripcion/up/MLAU165856224#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=44&amp;type=product&amp;tracking_id=2e8365dc-0eb4-4a06-b376-8750fa5af709&amp;wid=MLA1470455752&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Repuestos jancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>MLA1390286069</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Lote De 3 Libros Ediciones Selectas Y Grandes Exitos Orbis</t>
+        </is>
+      </c>
+      <c r="C442" t="n">
+        <v>11300</v>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.ar/lote-de-3-libros-ediciones-selectas-y-grandes-exitos-orbis/up/MLAU182269562#polycard_client=search-web-mobile&amp;be_origin=backend&amp;search_layout=stack&amp;position=45&amp;type=product&amp;tracking_id=2e8365dc-0eb4-4a06-b376-8750fa5af709&amp;wid=MLA1390286069&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
         <is>
           <t>Repuestos jancar</t>
         </is>

</xml_diff>